<commit_message>
Fix stage attribution by updating cached label on input actions
Instead of using current stage in AppendActual (which causes late output to be misattributed), update the _clientStartStageLabel when sending input. This ensures output from input responses is attributed to the input stage, not the start stage.

Also discovered: TC01_Empty test template has an Input action but it's not being executed by the grader, causing test failure.

Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SampleTestKitsWithData/Testkit_TCP_3/header.xlsx
+++ b/SampleTestKitsWithData/Testkit_TCP_3/header.xlsx
@@ -1,137 +1,62 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AB1ABE3-284B-4117-BA97-23BBB20364A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DataPattern" sheetId="3" r:id="rId1"/>
-    <sheet name="QuestionMark" sheetId="4" r:id="rId2"/>
-    <sheet name="TestSuite" sheetId="1" r:id="rId3"/>
-    <sheet name="Config" sheetId="5" r:id="rId4"/>
+    <sheet name="DataPattern" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="QuestionMark" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TestSuite" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Config" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
-  <si>
-    <t>Data Type</t>
-  </si>
-  <si>
-    <t>Pattern</t>
-  </si>
-  <si>
-    <t>Datetime</t>
-  </si>
-  <si>
-    <t>dd/MM/yyyy</t>
-  </si>
-  <si>
-    <t>Cases</t>
-  </si>
-  <si>
-    <t>Mark</t>
-  </si>
-  <si>
-    <t>TestCaseID</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Key</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Protocol</t>
-  </si>
-  <si>
-    <t>Console</t>
-  </si>
-  <si>
-    <t>TCP</t>
-  </si>
-  <si>
-    <t>TC01_Empty</t>
-  </si>
-  <si>
-    <t>TC02_ServerError</t>
-  </si>
-  <si>
-    <t>TC03_FullData</t>
-  </si>
-  <si>
-    <t>TC04_NoOrder</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="5">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -168,29 +93,88 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -456,31 +440,43 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="18.296875" customWidth="1"/>
-    <col min="2" max="2" width="22.19921875" customWidth="1"/>
-    <col min="3" max="3" width="21.8984375" customWidth="1"/>
+    <col width="18.296875" customWidth="1" min="1" max="1"/>
+    <col width="22.19921875" customWidth="1" min="2" max="2"/>
+    <col width="21.8984375" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="3"/>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Datetime</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>dd/MM/yyyy</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -488,50 +484,66 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="4" t="s">
+    <row r="1" customFormat="1" s="5">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Cases</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Mark</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC01_Empty</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC02_ServerError</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC03_FullData</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC04_NoOrder</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -541,92 +553,123 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.8984375" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="15.796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44.296875" style="5" customWidth="1"/>
-    <col min="3" max="4" width="8.8984375" style="5" customWidth="1"/>
-    <col min="5" max="16384" width="8.8984375" style="5"/>
+    <col width="15.796875" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
+    <col width="44.296875" customWidth="1" style="5" min="2" max="2"/>
+    <col width="8.8984375" customWidth="1" style="5" min="3" max="4"/>
+    <col width="8.8984375" customWidth="1" style="5" min="5" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2">
+    <row r="1" ht="13.5" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>TestCaseID</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC01_Empty</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC02_ServerError</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC03_FullData</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC04_NoOrder</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9C6C48B-55C0-4A7D-A267-4474B31A4631}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
-    <col min="2" max="2" width="10.296875" bestFit="1" customWidth="1"/>
+    <col width="10.296875" bestFit="1" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
+    <row r="1" customFormat="1" s="5">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Console</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>